<commit_message>
final touches b1 comparisons and title panel. started about
</commit_message>
<xml_diff>
--- a/Metadata/Metadata_YSI/YSI-metadata.xlsx
+++ b/Metadata/Metadata_YSI/YSI-metadata.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10212"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10609"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/grambihler/Documents/Data/GitHub/OceanWaterQuality/YSIExoSonde/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/grambihler/Documents/OceanWaterQuality/Metadata/Metadata_YSI/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9B3C2087-2FB6-D544-994C-E364E352E0C4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{89D6382C-94EA-B64C-83B2-5E95715CFE1F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-29840" yWindow="2840" windowWidth="28040" windowHeight="17180" activeTab="2" xr2:uid="{CB8DB564-CFB0-F34C-9A68-AB64D7227CFF}"/>
+    <workbookView xWindow="0" yWindow="500" windowWidth="68800" windowHeight="28300" xr2:uid="{CB8DB564-CFB0-F34C-9A68-AB64D7227CFF}"/>
   </bookViews>
   <sheets>
     <sheet name="Metadata" sheetId="1" r:id="rId1"/>
@@ -583,9 +583,6 @@
     <t>Data_Source_File</t>
   </si>
   <si>
-    <t>YSI ?</t>
-  </si>
-  <si>
     <t>?</t>
   </si>
   <si>
@@ -611,6 +608,9 @@
   </si>
   <si>
     <t>Chlorophyll</t>
+  </si>
+  <si>
+    <t>YSI 6600 V2</t>
   </si>
 </sst>
 </file>
@@ -747,9 +747,9 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office 2013 - 2022 Theme">
   <a:themeElements>
-    <a:clrScheme name="Office">
+    <a:clrScheme name="Office 2013 - 2022">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -787,7 +787,7 @@
         <a:srgbClr val="954F72"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office">
+    <a:fontScheme name="Office 2013 - 2022">
       <a:majorFont>
         <a:latin typeface="Calibri Light" panose="020F0302020204030204"/>
         <a:ea typeface=""/>
@@ -893,7 +893,7 @@
         <a:font script="Tfng" typeface="Ebrima"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office">
+    <a:fmtScheme name="Office 2013 - 2022">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -1035,7 +1035,7 @@
   <a:extraClrSchemeLst/>
   <a:extLst>
     <a:ext uri="{05A4C25C-085E-4340-85A3-A5531E510DB2}">
-      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
+      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office 2013 - 2022 Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
     </a:ext>
   </a:extLst>
 </a:theme>
@@ -1149,7 +1149,7 @@
         <v>172</v>
       </c>
       <c r="H2" s="5" t="s">
-        <v>182</v>
+        <v>181</v>
       </c>
       <c r="I2" t="s">
         <v>175</v>
@@ -1173,7 +1173,7 @@
         <v>4</v>
       </c>
       <c r="C3" t="s">
-        <v>186</v>
+        <v>185</v>
       </c>
       <c r="D3" t="s">
         <v>38</v>
@@ -1188,7 +1188,7 @@
         <v>172</v>
       </c>
       <c r="H3" s="5" t="s">
-        <v>182</v>
+        <v>181</v>
       </c>
       <c r="I3" t="s">
         <v>175</v>
@@ -1208,7 +1208,7 @@
         <v>4</v>
       </c>
       <c r="C4" t="s">
-        <v>187</v>
+        <v>186</v>
       </c>
       <c r="D4" t="s">
         <v>38</v>
@@ -1223,7 +1223,7 @@
         <v>172</v>
       </c>
       <c r="H4" s="5" t="s">
-        <v>182</v>
+        <v>181</v>
       </c>
       <c r="I4" t="s">
         <v>175</v>
@@ -1271,7 +1271,7 @@
         <v>172</v>
       </c>
       <c r="H5" s="5" t="s">
-        <v>182</v>
+        <v>181</v>
       </c>
       <c r="I5" t="s">
         <v>175</v>
@@ -1319,7 +1319,7 @@
         <v>172</v>
       </c>
       <c r="H6" s="5" t="s">
-        <v>182</v>
+        <v>181</v>
       </c>
       <c r="I6" t="s">
         <v>175</v>
@@ -1367,7 +1367,7 @@
         <v>172</v>
       </c>
       <c r="H7" s="5" t="s">
-        <v>182</v>
+        <v>181</v>
       </c>
       <c r="I7" t="s">
         <v>175</v>
@@ -1415,7 +1415,7 @@
         <v>172</v>
       </c>
       <c r="H8" s="5" t="s">
-        <v>182</v>
+        <v>181</v>
       </c>
       <c r="I8" t="s">
         <v>175</v>
@@ -1445,7 +1445,7 @@
         <v>14</v>
       </c>
       <c r="B9" t="s">
-        <v>188</v>
+        <v>187</v>
       </c>
       <c r="C9" t="s">
         <v>24</v>
@@ -1463,7 +1463,7 @@
         <v>172</v>
       </c>
       <c r="H9" s="5" t="s">
-        <v>182</v>
+        <v>181</v>
       </c>
       <c r="I9" t="s">
         <v>175</v>
@@ -1493,7 +1493,7 @@
         <v>16</v>
       </c>
       <c r="B10" t="s">
-        <v>190</v>
+        <v>189</v>
       </c>
       <c r="C10" t="s">
         <v>96</v>
@@ -1511,7 +1511,7 @@
         <v>172</v>
       </c>
       <c r="H10" s="5" t="s">
-        <v>182</v>
+        <v>181</v>
       </c>
       <c r="I10" t="s">
         <v>175</v>
@@ -1564,7 +1564,7 @@
         <v>172</v>
       </c>
       <c r="H11" s="5" t="s">
-        <v>182</v>
+        <v>181</v>
       </c>
       <c r="I11" t="s">
         <v>175</v>
@@ -1599,7 +1599,7 @@
         <v>172</v>
       </c>
       <c r="H12" s="5" t="s">
-        <v>182</v>
+        <v>181</v>
       </c>
       <c r="I12" t="s">
         <v>175</v>
@@ -1634,7 +1634,7 @@
         <v>172</v>
       </c>
       <c r="H13" s="5" t="s">
-        <v>182</v>
+        <v>181</v>
       </c>
       <c r="I13" t="s">
         <v>175</v>
@@ -1651,7 +1651,7 @@
         <v>39</v>
       </c>
       <c r="B14" t="s">
-        <v>188</v>
+        <v>187</v>
       </c>
       <c r="C14" t="s">
         <v>26</v>
@@ -1668,8 +1668,8 @@
       <c r="G14" s="9" t="s">
         <v>45</v>
       </c>
-      <c r="H14" s="11" t="s">
-        <v>181</v>
+      <c r="H14" s="5" t="s">
+        <v>190</v>
       </c>
       <c r="I14" s="11" t="s">
         <v>176</v>
@@ -1680,7 +1680,7 @@
         <v>40</v>
       </c>
       <c r="B15" t="s">
-        <v>190</v>
+        <v>189</v>
       </c>
       <c r="C15" t="s">
         <v>96</v>
@@ -1697,8 +1697,8 @@
       <c r="G15" s="9" t="s">
         <v>45</v>
       </c>
-      <c r="H15" s="11" t="s">
-        <v>181</v>
+      <c r="H15" s="5" t="s">
+        <v>190</v>
       </c>
       <c r="I15" s="11" t="s">
         <v>176</v>
@@ -1726,8 +1726,8 @@
       <c r="G16" s="9" t="s">
         <v>45</v>
       </c>
-      <c r="H16" s="11" t="s">
-        <v>181</v>
+      <c r="H16" s="5" t="s">
+        <v>190</v>
       </c>
       <c r="I16" s="11" t="s">
         <v>176</v>
@@ -1755,8 +1755,8 @@
       <c r="G17" s="9" t="s">
         <v>45</v>
       </c>
-      <c r="H17" s="11" t="s">
-        <v>181</v>
+      <c r="H17" s="5" t="s">
+        <v>190</v>
       </c>
       <c r="I17" s="11" t="s">
         <v>176</v>
@@ -1784,8 +1784,8 @@
       <c r="G18" s="9" t="s">
         <v>45</v>
       </c>
-      <c r="H18" s="11" t="s">
-        <v>181</v>
+      <c r="H18" s="5" t="s">
+        <v>190</v>
       </c>
       <c r="I18" s="11" t="s">
         <v>176</v>
@@ -1813,8 +1813,8 @@
       <c r="G19" s="9" t="s">
         <v>45</v>
       </c>
-      <c r="H19" s="11" t="s">
-        <v>181</v>
+      <c r="H19" s="5" t="s">
+        <v>190</v>
       </c>
       <c r="I19" s="11" t="s">
         <v>176</v>
@@ -1828,7 +1828,7 @@
         <v>4</v>
       </c>
       <c r="C20" t="s">
-        <v>187</v>
+        <v>186</v>
       </c>
       <c r="D20" t="s">
         <v>72</v>
@@ -1842,8 +1842,8 @@
       <c r="G20" s="9" t="s">
         <v>45</v>
       </c>
-      <c r="H20" s="11" t="s">
-        <v>181</v>
+      <c r="H20" s="5" t="s">
+        <v>190</v>
       </c>
       <c r="I20" s="11" t="s">
         <v>176</v>
@@ -1872,7 +1872,7 @@
         <v>45</v>
       </c>
       <c r="H21" s="11" t="s">
-        <v>183</v>
+        <v>182</v>
       </c>
       <c r="I21" s="11" t="s">
         <v>176</v>
@@ -1901,7 +1901,7 @@
         <v>45</v>
       </c>
       <c r="H22" s="11" t="s">
-        <v>183</v>
+        <v>182</v>
       </c>
       <c r="I22" s="11" t="s">
         <v>176</v>
@@ -1912,7 +1912,7 @@
         <v>102</v>
       </c>
       <c r="B23" t="s">
-        <v>190</v>
+        <v>189</v>
       </c>
       <c r="C23" t="s">
         <v>24</v>
@@ -1930,7 +1930,7 @@
         <v>45</v>
       </c>
       <c r="H23" s="11" t="s">
-        <v>183</v>
+        <v>182</v>
       </c>
       <c r="I23" s="11" t="s">
         <v>176</v>
@@ -1959,7 +1959,7 @@
         <v>45</v>
       </c>
       <c r="H24" s="11" t="s">
-        <v>183</v>
+        <v>182</v>
       </c>
       <c r="I24" s="11" t="s">
         <v>176</v>
@@ -1988,7 +1988,7 @@
         <v>45</v>
       </c>
       <c r="H25" s="11" t="s">
-        <v>183</v>
+        <v>182</v>
       </c>
       <c r="I25" s="11" t="s">
         <v>176</v>
@@ -2017,7 +2017,7 @@
         <v>45</v>
       </c>
       <c r="H26" s="11" t="s">
-        <v>183</v>
+        <v>182</v>
       </c>
       <c r="I26" s="11" t="s">
         <v>176</v>
@@ -2046,7 +2046,7 @@
         <v>45</v>
       </c>
       <c r="H27" s="11" t="s">
-        <v>183</v>
+        <v>182</v>
       </c>
       <c r="I27" s="11" t="s">
         <v>176</v>
@@ -2075,7 +2075,7 @@
         <v>45</v>
       </c>
       <c r="H28" s="11" t="s">
-        <v>183</v>
+        <v>182</v>
       </c>
       <c r="I28" s="11" t="s">
         <v>176</v>
@@ -2104,7 +2104,7 @@
         <v>45</v>
       </c>
       <c r="H29" s="11" t="s">
-        <v>183</v>
+        <v>182</v>
       </c>
       <c r="I29" s="11" t="s">
         <v>176</v>
@@ -2133,7 +2133,7 @@
         <v>45</v>
       </c>
       <c r="H30" s="11" t="s">
-        <v>183</v>
+        <v>182</v>
       </c>
       <c r="I30" s="11" t="s">
         <v>176</v>
@@ -2162,7 +2162,7 @@
         <v>45</v>
       </c>
       <c r="H31" s="11" t="s">
-        <v>183</v>
+        <v>182</v>
       </c>
       <c r="I31" s="11" t="s">
         <v>176</v>
@@ -2191,7 +2191,7 @@
         <v>45</v>
       </c>
       <c r="H32" s="11" t="s">
-        <v>183</v>
+        <v>182</v>
       </c>
       <c r="I32" s="11" t="s">
         <v>176</v>
@@ -2220,7 +2220,7 @@
         <v>45</v>
       </c>
       <c r="H33" s="11" t="s">
-        <v>183</v>
+        <v>182</v>
       </c>
       <c r="I33" s="11" t="s">
         <v>176</v>
@@ -2231,7 +2231,7 @@
         <v>118</v>
       </c>
       <c r="B34" t="s">
-        <v>188</v>
+        <v>187</v>
       </c>
       <c r="C34" t="s">
         <v>24</v>
@@ -2249,7 +2249,7 @@
         <v>45</v>
       </c>
       <c r="H34" s="11" t="s">
-        <v>183</v>
+        <v>182</v>
       </c>
       <c r="I34" s="11" t="s">
         <v>176</v>
@@ -2278,7 +2278,7 @@
         <v>45</v>
       </c>
       <c r="H35" s="11" t="s">
-        <v>183</v>
+        <v>182</v>
       </c>
       <c r="I35" s="11" t="s">
         <v>176</v>
@@ -2286,13 +2286,13 @@
     </row>
     <row r="36" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A36" t="s">
-        <v>185</v>
+        <v>184</v>
       </c>
       <c r="B36" t="s">
         <v>4</v>
       </c>
       <c r="C36" t="s">
-        <v>187</v>
+        <v>186</v>
       </c>
       <c r="D36" t="s">
         <v>63</v>
@@ -2307,7 +2307,7 @@
         <v>45</v>
       </c>
       <c r="H36" s="11" t="s">
-        <v>183</v>
+        <v>182</v>
       </c>
       <c r="I36" s="11" t="s">
         <v>176</v>
@@ -2315,13 +2315,13 @@
     </row>
     <row r="37" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A37" t="s">
-        <v>184</v>
+        <v>183</v>
       </c>
       <c r="B37" t="s">
         <v>4</v>
       </c>
       <c r="C37" t="s">
-        <v>186</v>
+        <v>185</v>
       </c>
       <c r="D37" t="s">
         <v>64</v>
@@ -2336,7 +2336,7 @@
         <v>45</v>
       </c>
       <c r="H37" s="11" t="s">
-        <v>183</v>
+        <v>182</v>
       </c>
       <c r="I37" s="11" t="s">
         <v>176</v>
@@ -2365,7 +2365,7 @@
         <v>45</v>
       </c>
       <c r="H38" s="11" t="s">
-        <v>183</v>
+        <v>182</v>
       </c>
       <c r="I38" s="11" t="s">
         <v>176</v>
@@ -2394,7 +2394,7 @@
         <v>46</v>
       </c>
       <c r="H39" s="11" t="s">
-        <v>183</v>
+        <v>182</v>
       </c>
       <c r="I39" s="11" t="s">
         <v>176</v>
@@ -2423,7 +2423,7 @@
         <v>46</v>
       </c>
       <c r="H40" s="11" t="s">
-        <v>183</v>
+        <v>182</v>
       </c>
       <c r="I40" s="11" t="s">
         <v>176</v>
@@ -2434,7 +2434,7 @@
         <v>102</v>
       </c>
       <c r="B41" t="s">
-        <v>190</v>
+        <v>189</v>
       </c>
       <c r="C41" t="s">
         <v>24</v>
@@ -2452,7 +2452,7 @@
         <v>46</v>
       </c>
       <c r="H41" s="11" t="s">
-        <v>183</v>
+        <v>182</v>
       </c>
       <c r="I41" s="11" t="s">
         <v>176</v>
@@ -2481,7 +2481,7 @@
         <v>46</v>
       </c>
       <c r="H42" s="11" t="s">
-        <v>183</v>
+        <v>182</v>
       </c>
       <c r="I42" s="11" t="s">
         <v>176</v>
@@ -2510,7 +2510,7 @@
         <v>46</v>
       </c>
       <c r="H43" s="11" t="s">
-        <v>183</v>
+        <v>182</v>
       </c>
       <c r="I43" s="11" t="s">
         <v>176</v>
@@ -2539,7 +2539,7 @@
         <v>46</v>
       </c>
       <c r="H44" s="11" t="s">
-        <v>183</v>
+        <v>182</v>
       </c>
       <c r="I44" s="11" t="s">
         <v>176</v>
@@ -2568,7 +2568,7 @@
         <v>46</v>
       </c>
       <c r="H45" s="11" t="s">
-        <v>183</v>
+        <v>182</v>
       </c>
       <c r="I45" s="11" t="s">
         <v>176</v>
@@ -2597,7 +2597,7 @@
         <v>46</v>
       </c>
       <c r="H46" s="11" t="s">
-        <v>183</v>
+        <v>182</v>
       </c>
       <c r="I46" s="11" t="s">
         <v>176</v>
@@ -2626,7 +2626,7 @@
         <v>46</v>
       </c>
       <c r="H47" s="11" t="s">
-        <v>183</v>
+        <v>182</v>
       </c>
       <c r="I47" s="11" t="s">
         <v>176</v>
@@ -2655,7 +2655,7 @@
         <v>46</v>
       </c>
       <c r="H48" s="11" t="s">
-        <v>183</v>
+        <v>182</v>
       </c>
       <c r="I48" s="11" t="s">
         <v>176</v>
@@ -2684,7 +2684,7 @@
         <v>46</v>
       </c>
       <c r="H49" s="11" t="s">
-        <v>183</v>
+        <v>182</v>
       </c>
       <c r="I49" s="11" t="s">
         <v>176</v>
@@ -2713,7 +2713,7 @@
         <v>46</v>
       </c>
       <c r="H50" s="11" t="s">
-        <v>183</v>
+        <v>182</v>
       </c>
       <c r="I50" s="11" t="s">
         <v>176</v>
@@ -2742,7 +2742,7 @@
         <v>46</v>
       </c>
       <c r="H51" s="11" t="s">
-        <v>183</v>
+        <v>182</v>
       </c>
       <c r="I51" s="11" t="s">
         <v>176</v>
@@ -2771,7 +2771,7 @@
         <v>46</v>
       </c>
       <c r="H52" s="11" t="s">
-        <v>183</v>
+        <v>182</v>
       </c>
       <c r="I52" s="11" t="s">
         <v>176</v>
@@ -2782,7 +2782,7 @@
         <v>118</v>
       </c>
       <c r="B53" t="s">
-        <v>188</v>
+        <v>187</v>
       </c>
       <c r="C53" t="s">
         <v>24</v>
@@ -2800,7 +2800,7 @@
         <v>46</v>
       </c>
       <c r="H53" s="11" t="s">
-        <v>183</v>
+        <v>182</v>
       </c>
       <c r="I53" s="11" t="s">
         <v>176</v>
@@ -2829,7 +2829,7 @@
         <v>46</v>
       </c>
       <c r="H54" s="11" t="s">
-        <v>183</v>
+        <v>182</v>
       </c>
       <c r="I54" s="11" t="s">
         <v>176</v>
@@ -2837,13 +2837,13 @@
     </row>
     <row r="55" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A55" t="s">
-        <v>185</v>
+        <v>184</v>
       </c>
       <c r="B55" t="s">
         <v>4</v>
       </c>
       <c r="C55" t="s">
-        <v>187</v>
+        <v>186</v>
       </c>
       <c r="D55" t="s">
         <v>89</v>
@@ -2858,7 +2858,7 @@
         <v>46</v>
       </c>
       <c r="H55" s="11" t="s">
-        <v>183</v>
+        <v>182</v>
       </c>
       <c r="I55" s="11" t="s">
         <v>176</v>
@@ -2866,13 +2866,13 @@
     </row>
     <row r="56" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A56" t="s">
-        <v>184</v>
+        <v>183</v>
       </c>
       <c r="B56" t="s">
         <v>4</v>
       </c>
       <c r="C56" t="s">
-        <v>186</v>
+        <v>185</v>
       </c>
       <c r="D56" t="s">
         <v>90</v>
@@ -2887,7 +2887,7 @@
         <v>46</v>
       </c>
       <c r="H56" s="11" t="s">
-        <v>183</v>
+        <v>182</v>
       </c>
       <c r="I56" s="11" t="s">
         <v>176</v>
@@ -2916,7 +2916,7 @@
         <v>46</v>
       </c>
       <c r="H57" s="11" t="s">
-        <v>183</v>
+        <v>182</v>
       </c>
       <c r="I57" s="11" t="s">
         <v>176</v>
@@ -2945,7 +2945,7 @@
         <v>46</v>
       </c>
       <c r="H58" s="11" t="s">
-        <v>183</v>
+        <v>182</v>
       </c>
       <c r="I58" s="11" t="s">
         <v>176</v>
@@ -2974,7 +2974,7 @@
         <v>172</v>
       </c>
       <c r="H59" s="5" t="s">
-        <v>181</v>
+        <v>190</v>
       </c>
       <c r="I59" s="12" t="s">
         <v>177</v>
@@ -2985,7 +2985,7 @@
         <v>157</v>
       </c>
       <c r="B60" t="s">
-        <v>190</v>
+        <v>189</v>
       </c>
       <c r="C60" t="s">
         <v>96</v>
@@ -3003,7 +3003,7 @@
         <v>172</v>
       </c>
       <c r="H60" s="5" t="s">
-        <v>181</v>
+        <v>190</v>
       </c>
       <c r="I60" s="12" t="s">
         <v>177</v>
@@ -3014,7 +3014,7 @@
         <v>156</v>
       </c>
       <c r="B61" t="s">
-        <v>188</v>
+        <v>187</v>
       </c>
       <c r="C61" t="s">
         <v>26</v>
@@ -3032,7 +3032,7 @@
         <v>172</v>
       </c>
       <c r="H61" s="5" t="s">
-        <v>181</v>
+        <v>190</v>
       </c>
       <c r="I61" s="12" t="s">
         <v>177</v>
@@ -3061,7 +3061,7 @@
         <v>172</v>
       </c>
       <c r="H62" s="5" t="s">
-        <v>181</v>
+        <v>190</v>
       </c>
       <c r="I62" s="12" t="s">
         <v>177</v>
@@ -3090,7 +3090,7 @@
         <v>172</v>
       </c>
       <c r="H63" s="5" t="s">
-        <v>181</v>
+        <v>190</v>
       </c>
       <c r="I63" s="12" t="s">
         <v>177</v>
@@ -3119,7 +3119,7 @@
         <v>172</v>
       </c>
       <c r="H64" s="5" t="s">
-        <v>181</v>
+        <v>190</v>
       </c>
       <c r="I64" s="12" t="s">
         <v>177</v>
@@ -3148,7 +3148,7 @@
         <v>172</v>
       </c>
       <c r="H65" s="5" t="s">
-        <v>181</v>
+        <v>190</v>
       </c>
       <c r="I65" s="12" t="s">
         <v>177</v>
@@ -3162,7 +3162,7 @@
         <v>4</v>
       </c>
       <c r="C66" t="s">
-        <v>187</v>
+        <v>186</v>
       </c>
       <c r="D66" t="s">
         <v>143</v>
@@ -3177,7 +3177,7 @@
         <v>172</v>
       </c>
       <c r="H66" s="5" t="s">
-        <v>181</v>
+        <v>190</v>
       </c>
       <c r="I66" s="12" t="s">
         <v>177</v>
@@ -3206,7 +3206,7 @@
         <v>172</v>
       </c>
       <c r="H67" s="5" t="s">
-        <v>181</v>
+        <v>190</v>
       </c>
       <c r="I67" s="12" t="s">
         <v>177</v>
@@ -3235,7 +3235,7 @@
         <v>172</v>
       </c>
       <c r="H68" s="5" t="s">
-        <v>181</v>
+        <v>190</v>
       </c>
       <c r="I68" s="12" t="s">
         <v>177</v>
@@ -3264,7 +3264,7 @@
         <v>172</v>
       </c>
       <c r="H69" s="5" t="s">
-        <v>181</v>
+        <v>190</v>
       </c>
       <c r="I69" s="12" t="s">
         <v>177</v>
@@ -3275,7 +3275,7 @@
         <v>157</v>
       </c>
       <c r="B70" t="s">
-        <v>190</v>
+        <v>189</v>
       </c>
       <c r="C70" t="s">
         <v>96</v>
@@ -3293,7 +3293,7 @@
         <v>172</v>
       </c>
       <c r="H70" s="5" t="s">
-        <v>181</v>
+        <v>190</v>
       </c>
       <c r="I70" s="12" t="s">
         <v>177</v>
@@ -3304,7 +3304,7 @@
         <v>156</v>
       </c>
       <c r="B71" t="s">
-        <v>188</v>
+        <v>187</v>
       </c>
       <c r="C71" t="s">
         <v>26</v>
@@ -3322,7 +3322,7 @@
         <v>172</v>
       </c>
       <c r="H71" s="5" t="s">
-        <v>181</v>
+        <v>190</v>
       </c>
       <c r="I71" s="12" t="s">
         <v>177</v>
@@ -3351,7 +3351,7 @@
         <v>172</v>
       </c>
       <c r="H72" s="5" t="s">
-        <v>181</v>
+        <v>190</v>
       </c>
       <c r="I72" s="12" t="s">
         <v>177</v>
@@ -3380,7 +3380,7 @@
         <v>172</v>
       </c>
       <c r="H73" s="5" t="s">
-        <v>181</v>
+        <v>190</v>
       </c>
       <c r="I73" s="12" t="s">
         <v>177</v>
@@ -3409,7 +3409,7 @@
         <v>172</v>
       </c>
       <c r="H74" s="5" t="s">
-        <v>181</v>
+        <v>190</v>
       </c>
       <c r="I74" s="12" t="s">
         <v>177</v>
@@ -3438,7 +3438,7 @@
         <v>172</v>
       </c>
       <c r="H75" s="5" t="s">
-        <v>181</v>
+        <v>190</v>
       </c>
       <c r="I75" s="12" t="s">
         <v>177</v>
@@ -3452,7 +3452,7 @@
         <v>4</v>
       </c>
       <c r="C76" t="s">
-        <v>187</v>
+        <v>186</v>
       </c>
       <c r="D76" t="s">
         <v>144</v>
@@ -3467,7 +3467,7 @@
         <v>172</v>
       </c>
       <c r="H76" s="5" t="s">
-        <v>181</v>
+        <v>190</v>
       </c>
       <c r="I76" s="12" t="s">
         <v>177</v>
@@ -3496,7 +3496,7 @@
         <v>172</v>
       </c>
       <c r="H77" s="5" t="s">
-        <v>182</v>
+        <v>181</v>
       </c>
       <c r="I77" s="12" t="s">
         <v>177</v>
@@ -3510,7 +3510,7 @@
         <v>160</v>
       </c>
       <c r="C78" t="s">
-        <v>186</v>
+        <v>185</v>
       </c>
       <c r="D78" t="s">
         <v>142</v>
@@ -3525,7 +3525,7 @@
         <v>172</v>
       </c>
       <c r="H78" s="5" t="s">
-        <v>182</v>
+        <v>181</v>
       </c>
       <c r="I78" s="12" t="s">
         <v>177</v>
@@ -3539,7 +3539,7 @@
         <v>4</v>
       </c>
       <c r="C79" t="s">
-        <v>187</v>
+        <v>186</v>
       </c>
       <c r="D79" t="s">
         <v>142</v>
@@ -3554,7 +3554,7 @@
         <v>172</v>
       </c>
       <c r="H79" s="5" t="s">
-        <v>182</v>
+        <v>181</v>
       </c>
       <c r="I79" s="12" t="s">
         <v>177</v>
@@ -3583,7 +3583,7 @@
         <v>172</v>
       </c>
       <c r="H80" s="5" t="s">
-        <v>182</v>
+        <v>181</v>
       </c>
       <c r="I80" s="12" t="s">
         <v>177</v>
@@ -3612,7 +3612,7 @@
         <v>172</v>
       </c>
       <c r="H81" s="5" t="s">
-        <v>182</v>
+        <v>181</v>
       </c>
       <c r="I81" s="12" t="s">
         <v>177</v>
@@ -3641,7 +3641,7 @@
         <v>172</v>
       </c>
       <c r="H82" s="5" t="s">
-        <v>182</v>
+        <v>181</v>
       </c>
       <c r="I82" s="12" t="s">
         <v>177</v>
@@ -3670,7 +3670,7 @@
         <v>172</v>
       </c>
       <c r="H83" s="5" t="s">
-        <v>182</v>
+        <v>181</v>
       </c>
       <c r="I83" s="12" t="s">
         <v>177</v>
@@ -3699,7 +3699,7 @@
         <v>172</v>
       </c>
       <c r="H84" s="5" t="s">
-        <v>182</v>
+        <v>181</v>
       </c>
       <c r="I84" s="12" t="s">
         <v>177</v>
@@ -3713,7 +3713,7 @@
         <v>160</v>
       </c>
       <c r="C85" t="s">
-        <v>186</v>
+        <v>185</v>
       </c>
       <c r="D85" t="s">
         <v>148</v>
@@ -3728,7 +3728,7 @@
         <v>172</v>
       </c>
       <c r="H85" s="5" t="s">
-        <v>182</v>
+        <v>181</v>
       </c>
       <c r="I85" s="12" t="s">
         <v>177</v>
@@ -3742,7 +3742,7 @@
         <v>4</v>
       </c>
       <c r="C86" t="s">
-        <v>187</v>
+        <v>186</v>
       </c>
       <c r="D86" t="s">
         <v>148</v>
@@ -3757,7 +3757,7 @@
         <v>172</v>
       </c>
       <c r="H86" s="5" t="s">
-        <v>182</v>
+        <v>181</v>
       </c>
       <c r="I86" s="12" t="s">
         <v>177</v>
@@ -3786,7 +3786,7 @@
         <v>172</v>
       </c>
       <c r="H87" s="5" t="s">
-        <v>182</v>
+        <v>181</v>
       </c>
       <c r="I87" s="12" t="s">
         <v>177</v>
@@ -3815,7 +3815,7 @@
         <v>172</v>
       </c>
       <c r="H88" s="5" t="s">
-        <v>182</v>
+        <v>181</v>
       </c>
       <c r="I88" s="12" t="s">
         <v>177</v>
@@ -3844,7 +3844,7 @@
         <v>172</v>
       </c>
       <c r="H89" s="5" t="s">
-        <v>182</v>
+        <v>181</v>
       </c>
       <c r="I89" s="12" t="s">
         <v>177</v>
@@ -3873,7 +3873,7 @@
         <v>172</v>
       </c>
       <c r="H90" s="5" t="s">
-        <v>182</v>
+        <v>181</v>
       </c>
       <c r="I90" s="12" t="s">
         <v>177</v>
@@ -3902,7 +3902,7 @@
         <v>172</v>
       </c>
       <c r="H91" s="5" t="s">
-        <v>182</v>
+        <v>181</v>
       </c>
       <c r="I91" s="12" t="s">
         <v>177</v>
@@ -3916,7 +3916,7 @@
         <v>160</v>
       </c>
       <c r="C92" t="s">
-        <v>186</v>
+        <v>185</v>
       </c>
       <c r="D92" t="s">
         <v>138</v>
@@ -3931,7 +3931,7 @@
         <v>172</v>
       </c>
       <c r="H92" s="5" t="s">
-        <v>182</v>
+        <v>181</v>
       </c>
       <c r="I92" s="12" t="s">
         <v>177</v>
@@ -3945,7 +3945,7 @@
         <v>4</v>
       </c>
       <c r="C93" t="s">
-        <v>187</v>
+        <v>186</v>
       </c>
       <c r="D93" t="s">
         <v>138</v>
@@ -3960,7 +3960,7 @@
         <v>172</v>
       </c>
       <c r="H93" s="5" t="s">
-        <v>182</v>
+        <v>181</v>
       </c>
       <c r="I93" s="12" t="s">
         <v>177</v>
@@ -3989,7 +3989,7 @@
         <v>172</v>
       </c>
       <c r="H94" s="5" t="s">
-        <v>182</v>
+        <v>181</v>
       </c>
       <c r="I94" s="12" t="s">
         <v>177</v>
@@ -4018,7 +4018,7 @@
         <v>172</v>
       </c>
       <c r="H95" s="5" t="s">
-        <v>182</v>
+        <v>181</v>
       </c>
       <c r="I95" s="12" t="s">
         <v>177</v>
@@ -4047,7 +4047,7 @@
         <v>172</v>
       </c>
       <c r="H96" s="5" t="s">
-        <v>182</v>
+        <v>181</v>
       </c>
       <c r="I96" s="12" t="s">
         <v>177</v>
@@ -4076,7 +4076,7 @@
         <v>172</v>
       </c>
       <c r="H97" s="5" t="s">
-        <v>182</v>
+        <v>181</v>
       </c>
       <c r="I97" s="12" t="s">
         <v>177</v>
@@ -4105,7 +4105,7 @@
         <v>172</v>
       </c>
       <c r="H98" s="5" t="s">
-        <v>182</v>
+        <v>181</v>
       </c>
       <c r="I98" s="12" t="s">
         <v>177</v>
@@ -4119,7 +4119,7 @@
         <v>160</v>
       </c>
       <c r="C99" t="s">
-        <v>186</v>
+        <v>185</v>
       </c>
       <c r="D99" t="s">
         <v>137</v>
@@ -4134,7 +4134,7 @@
         <v>172</v>
       </c>
       <c r="H99" s="5" t="s">
-        <v>182</v>
+        <v>181</v>
       </c>
       <c r="I99" s="12" t="s">
         <v>177</v>
@@ -4148,7 +4148,7 @@
         <v>4</v>
       </c>
       <c r="C100" t="s">
-        <v>187</v>
+        <v>186</v>
       </c>
       <c r="D100" t="s">
         <v>137</v>
@@ -4163,7 +4163,7 @@
         <v>172</v>
       </c>
       <c r="H100" s="5" t="s">
-        <v>182</v>
+        <v>181</v>
       </c>
       <c r="I100" s="12" t="s">
         <v>177</v>
@@ -4192,7 +4192,7 @@
         <v>172</v>
       </c>
       <c r="H101" s="5" t="s">
-        <v>182</v>
+        <v>181</v>
       </c>
       <c r="I101" s="12" t="s">
         <v>177</v>
@@ -4221,7 +4221,7 @@
         <v>172</v>
       </c>
       <c r="H102" s="5" t="s">
-        <v>182</v>
+        <v>181</v>
       </c>
       <c r="I102" s="12" t="s">
         <v>177</v>
@@ -4250,7 +4250,7 @@
         <v>172</v>
       </c>
       <c r="H103" s="5" t="s">
-        <v>182</v>
+        <v>181</v>
       </c>
       <c r="I103" s="12" t="s">
         <v>177</v>
@@ -4279,7 +4279,7 @@
         <v>172</v>
       </c>
       <c r="H104" s="5" t="s">
-        <v>182</v>
+        <v>181</v>
       </c>
       <c r="I104" s="12" t="s">
         <v>177</v>
@@ -4290,7 +4290,7 @@
         <v>166</v>
       </c>
       <c r="B105" t="s">
-        <v>188</v>
+        <v>187</v>
       </c>
       <c r="C105" t="s">
         <v>24</v>
@@ -4308,7 +4308,7 @@
         <v>172</v>
       </c>
       <c r="H105" s="5" t="s">
-        <v>182</v>
+        <v>181</v>
       </c>
       <c r="I105" s="12" t="s">
         <v>177</v>
@@ -4319,7 +4319,7 @@
         <v>167</v>
       </c>
       <c r="B106" t="s">
-        <v>190</v>
+        <v>189</v>
       </c>
       <c r="C106" t="s">
         <v>96</v>
@@ -4337,7 +4337,7 @@
         <v>172</v>
       </c>
       <c r="H106" s="5" t="s">
-        <v>182</v>
+        <v>181</v>
       </c>
       <c r="I106" s="12" t="s">
         <v>177</v>
@@ -4366,7 +4366,7 @@
         <v>172</v>
       </c>
       <c r="H107" s="5" t="s">
-        <v>182</v>
+        <v>181</v>
       </c>
       <c r="I107" s="12" t="s">
         <v>177</v>
@@ -4395,7 +4395,7 @@
         <v>172</v>
       </c>
       <c r="H108" s="5" t="s">
-        <v>182</v>
+        <v>181</v>
       </c>
       <c r="I108" s="12" t="s">
         <v>177</v>
@@ -4409,7 +4409,7 @@
         <v>160</v>
       </c>
       <c r="C109" t="s">
-        <v>186</v>
+        <v>185</v>
       </c>
       <c r="D109" t="s">
         <v>139</v>
@@ -4424,7 +4424,7 @@
         <v>172</v>
       </c>
       <c r="H109" s="5" t="s">
-        <v>182</v>
+        <v>181</v>
       </c>
       <c r="I109" s="12" t="s">
         <v>177</v>
@@ -4438,7 +4438,7 @@
         <v>4</v>
       </c>
       <c r="C110" t="s">
-        <v>187</v>
+        <v>186</v>
       </c>
       <c r="D110" t="s">
         <v>139</v>
@@ -4453,7 +4453,7 @@
         <v>172</v>
       </c>
       <c r="H110" s="5" t="s">
-        <v>182</v>
+        <v>181</v>
       </c>
       <c r="I110" s="12" t="s">
         <v>177</v>
@@ -4482,7 +4482,7 @@
         <v>172</v>
       </c>
       <c r="H111" s="5" t="s">
-        <v>182</v>
+        <v>181</v>
       </c>
       <c r="I111" s="12" t="s">
         <v>177</v>
@@ -4511,7 +4511,7 @@
         <v>172</v>
       </c>
       <c r="H112" s="5" t="s">
-        <v>182</v>
+        <v>181</v>
       </c>
       <c r="I112" s="12" t="s">
         <v>177</v>
@@ -4540,7 +4540,7 @@
         <v>172</v>
       </c>
       <c r="H113" s="5" t="s">
-        <v>182</v>
+        <v>181</v>
       </c>
       <c r="I113" s="12" t="s">
         <v>177</v>
@@ -4569,7 +4569,7 @@
         <v>172</v>
       </c>
       <c r="H114" s="5" t="s">
-        <v>182</v>
+        <v>181</v>
       </c>
       <c r="I114" s="12" t="s">
         <v>177</v>
@@ -4598,7 +4598,7 @@
         <v>172</v>
       </c>
       <c r="H115" s="5" t="s">
-        <v>182</v>
+        <v>181</v>
       </c>
       <c r="I115" s="12" t="s">
         <v>177</v>
@@ -4612,7 +4612,7 @@
         <v>160</v>
       </c>
       <c r="C116" t="s">
-        <v>186</v>
+        <v>185</v>
       </c>
       <c r="D116" t="s">
         <v>135</v>
@@ -4627,7 +4627,7 @@
         <v>172</v>
       </c>
       <c r="H116" s="5" t="s">
-        <v>182</v>
+        <v>181</v>
       </c>
       <c r="I116" s="12" t="s">
         <v>177</v>
@@ -4641,7 +4641,7 @@
         <v>4</v>
       </c>
       <c r="C117" t="s">
-        <v>187</v>
+        <v>186</v>
       </c>
       <c r="D117" t="s">
         <v>135</v>
@@ -4656,7 +4656,7 @@
         <v>172</v>
       </c>
       <c r="H117" s="5" t="s">
-        <v>182</v>
+        <v>181</v>
       </c>
       <c r="I117" s="12" t="s">
         <v>177</v>
@@ -4685,7 +4685,7 @@
         <v>172</v>
       </c>
       <c r="H118" s="5" t="s">
-        <v>182</v>
+        <v>181</v>
       </c>
       <c r="I118" s="12" t="s">
         <v>177</v>
@@ -4714,7 +4714,7 @@
         <v>172</v>
       </c>
       <c r="H119" s="5" t="s">
-        <v>182</v>
+        <v>181</v>
       </c>
       <c r="I119" s="12" t="s">
         <v>177</v>
@@ -4743,7 +4743,7 @@
         <v>172</v>
       </c>
       <c r="H120" s="5" t="s">
-        <v>182</v>
+        <v>181</v>
       </c>
       <c r="I120" s="12" t="s">
         <v>177</v>
@@ -4772,7 +4772,7 @@
         <v>172</v>
       </c>
       <c r="H121" s="5" t="s">
-        <v>182</v>
+        <v>181</v>
       </c>
       <c r="I121" s="12" t="s">
         <v>177</v>
@@ -4783,7 +4783,7 @@
         <v>169</v>
       </c>
       <c r="B122" t="s">
-        <v>188</v>
+        <v>187</v>
       </c>
       <c r="C122" t="s">
         <v>24</v>
@@ -4801,7 +4801,7 @@
         <v>172</v>
       </c>
       <c r="H122" s="5" t="s">
-        <v>182</v>
+        <v>181</v>
       </c>
       <c r="I122" s="12" t="s">
         <v>177</v>
@@ -4812,7 +4812,7 @@
         <v>170</v>
       </c>
       <c r="B123" t="s">
-        <v>189</v>
+        <v>188</v>
       </c>
       <c r="C123" t="s">
         <v>24</v>
@@ -4830,7 +4830,7 @@
         <v>172</v>
       </c>
       <c r="H123" s="5" t="s">
-        <v>182</v>
+        <v>181</v>
       </c>
       <c r="I123" s="12" t="s">
         <v>177</v>
@@ -4841,7 +4841,7 @@
         <v>171</v>
       </c>
       <c r="B124" t="s">
-        <v>190</v>
+        <v>189</v>
       </c>
       <c r="C124" t="s">
         <v>96</v>
@@ -4859,7 +4859,7 @@
         <v>172</v>
       </c>
       <c r="H124" s="5" t="s">
-        <v>182</v>
+        <v>181</v>
       </c>
       <c r="I124" s="12" t="s">
         <v>177</v>

</xml_diff>

<commit_message>
added in data that was previously missed. using different raw data files than before
</commit_message>
<xml_diff>
--- a/Metadata/Metadata_YSI/YSI-metadata.xlsx
+++ b/Metadata/Metadata_YSI/YSI-metadata.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/grambihler/Documents/OceanWaterQuality/Metadata/Metadata_YSI/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{89D6382C-94EA-B64C-83B2-5E95715CFE1F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{224E76CB-D547-C047-AADF-F2AA0FAD0229}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="500" windowWidth="68800" windowHeight="28300" xr2:uid="{CB8DB564-CFB0-F34C-9A68-AB64D7227CFF}"/>
+    <workbookView xWindow="0" yWindow="11820" windowWidth="68800" windowHeight="16980" activeTab="2" xr2:uid="{CB8DB564-CFB0-F34C-9A68-AB64D7227CFF}"/>
   </bookViews>
   <sheets>
     <sheet name="Metadata" sheetId="1" r:id="rId1"/>
@@ -11983,7 +11983,7 @@
       </c>
     </row>
     <row r="2" spans="1:14" x14ac:dyDescent="0.2">
-      <c r="A2" t="s">
+      <c r="A2" s="6" t="s">
         <v>142</v>
       </c>
       <c r="B2" s="3">
@@ -11996,7 +11996,7 @@
       </c>
     </row>
     <row r="3" spans="1:14" x14ac:dyDescent="0.2">
-      <c r="A3" t="s">
+      <c r="A3" s="6" t="s">
         <v>138</v>
       </c>
       <c r="B3" s="1"/>
@@ -12009,7 +12009,7 @@
       </c>
     </row>
     <row r="4" spans="1:14" x14ac:dyDescent="0.2">
-      <c r="A4" t="s">
+      <c r="A4" s="6" t="s">
         <v>139</v>
       </c>
       <c r="D4" s="1"/>
@@ -12043,7 +12043,7 @@
       </c>
     </row>
     <row r="7" spans="1:14" x14ac:dyDescent="0.2">
-      <c r="A7" t="s">
+      <c r="A7" s="6" t="s">
         <v>137</v>
       </c>
       <c r="G7" s="3">
@@ -12055,7 +12055,7 @@
       </c>
     </row>
     <row r="8" spans="1:14" x14ac:dyDescent="0.2">
-      <c r="A8" t="s">
+      <c r="A8" s="6" t="s">
         <v>137</v>
       </c>
       <c r="G8" s="1"/>
@@ -12064,7 +12064,7 @@
       </c>
     </row>
     <row r="9" spans="1:14" x14ac:dyDescent="0.2">
-      <c r="A9" t="s">
+      <c r="A9" s="6" t="s">
         <v>144</v>
       </c>
       <c r="G9" s="1"/>
@@ -12092,7 +12092,7 @@
       </c>
     </row>
     <row r="11" spans="1:14" x14ac:dyDescent="0.2">
-      <c r="A11" t="s">
+      <c r="A11" s="6" t="s">
         <v>137</v>
       </c>
       <c r="I11" s="3" t="s">

</xml_diff>